<commit_message>
Sync planning SharePoint : S29
</commit_message>
<xml_diff>
--- a/Plannings 2026 S29.xlsx
+++ b/Plannings 2026 S29.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8CF4306E-CBE7-4479-BF2B-A1EAC20E8DEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{8CF4306E-CBE7-4479-BF2B-A1EAC20E8DEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F2EAFFF2-A0B7-43AE-9B64-E6F33C87DBB7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -150,9 +150,6 @@
     <t>17:30/24:00</t>
   </si>
   <si>
-    <t>17:00/24:00</t>
-  </si>
-  <si>
     <t>10:00/18:00</t>
   </si>
   <si>
@@ -316,6 +313,9 @@
   </si>
   <si>
     <t>STAGE // P25M</t>
+  </si>
+  <si>
+    <t>18:00/24:00</t>
   </si>
 </sst>
 </file>
@@ -5002,19 +5002,19 @@
     </row>
     <row r="3" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B3" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C3" s="56" t="s">
+        <v>95</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="F3" s="15" t="s">
         <v>96</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>97</v>
       </c>
       <c r="G3" s="15"/>
       <c r="H3" s="15"/>
@@ -5297,7 +5297,7 @@
       </c>
       <c r="D20" s="21"/>
       <c r="E20" s="54" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F20" s="21" t="s">
         <v>14</v>
@@ -5313,23 +5313,23 @@
         <v>41</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>42</v>
+        <v>97</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="55" t="s">
+        <v>42</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="G21" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>45</v>
       </c>
       <c r="H21" s="28"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="20" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B22" s="21"/>
       <c r="C22" s="26"/>
@@ -5351,19 +5351,19 @@
       <c r="C23" s="24"/>
       <c r="D23" s="24"/>
       <c r="E23" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="F23" s="24" t="s">
         <v>47</v>
-      </c>
-      <c r="F23" s="24" t="s">
-        <v>48</v>
       </c>
       <c r="G23" s="24"/>
       <c r="H23" s="25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="40" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B24" s="41"/>
       <c r="C24" s="42"/>
@@ -5375,7 +5375,7 @@
     </row>
     <row r="25" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B25" s="30"/>
       <c r="C25" s="31"/>
@@ -5387,7 +5387,7 @@
     </row>
     <row r="26" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B26" s="30"/>
       <c r="C26" s="31"/>
@@ -5399,7 +5399,7 @@
     </row>
     <row r="27" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B27" s="30"/>
       <c r="C27" s="31"/>
@@ -5411,7 +5411,7 @@
     </row>
     <row r="28" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B28" s="30"/>
       <c r="C28" s="31"/>
@@ -5423,11 +5423,11 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B29" s="21"/>
       <c r="C29" s="48" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D29" s="21" t="s">
         <v>14</v>
@@ -5441,7 +5441,7 @@
       <c r="A30" s="23"/>
       <c r="B30" s="24"/>
       <c r="C30" s="50" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D30" s="24" t="s">
         <v>20</v>
@@ -5453,7 +5453,7 @@
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="20" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B31" s="21"/>
       <c r="C31" s="26"/>
@@ -5475,15 +5475,15 @@
       <c r="E32" s="24"/>
       <c r="F32" s="24"/>
       <c r="G32" s="24" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H32" s="25" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="16" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B33" s="30"/>
       <c r="C33" s="31"/>
@@ -5495,7 +5495,7 @@
     </row>
     <row r="34" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B34" s="30"/>
       <c r="C34" s="31"/>
@@ -5507,7 +5507,7 @@
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="35" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>14</v>
@@ -5517,10 +5517,10 @@
         <v>14</v>
       </c>
       <c r="E35" s="52" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F35" s="52" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G35" s="1"/>
       <c r="H35" s="28"/>
@@ -5528,17 +5528,17 @@
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="27"/>
       <c r="B36" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1" t="s">
         <v>15</v>
       </c>
       <c r="E36" s="52" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F36" s="52" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G36" s="1"/>
       <c r="H36" s="28"/>
@@ -5555,7 +5555,7 @@
     </row>
     <row r="38" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B38" s="30"/>
       <c r="C38" s="31"/>
@@ -5567,22 +5567,22 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="B39" s="44" t="s">
         <v>66</v>
       </c>
-      <c r="B39" s="44" t="s">
-        <v>67</v>
-      </c>
       <c r="C39" s="44" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D39" s="44" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E39" s="44" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F39" s="44" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G39" s="21"/>
       <c r="H39" s="22"/>
@@ -5590,19 +5590,19 @@
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="27"/>
       <c r="B40" s="45" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C40" s="45" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D40" s="45" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E40" s="45" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F40" s="45" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G40" s="1"/>
       <c r="H40" s="28"/>
@@ -5610,19 +5610,19 @@
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="27"/>
       <c r="B41" s="46" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C41" s="46" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D41" s="46" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E41" s="46" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F41" s="46" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G41" s="1"/>
       <c r="H41" s="28"/>
@@ -5630,19 +5630,19 @@
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="27"/>
       <c r="B42" s="45" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C42" s="45" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D42" s="45" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E42" s="45" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F42" s="45" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G42" s="1"/>
       <c r="H42" s="28"/>
@@ -5650,19 +5650,19 @@
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="27"/>
       <c r="B43" s="46" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C43" s="46" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D43" s="46" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E43" s="46" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F43" s="46" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G43" s="1"/>
       <c r="H43" s="28"/>
@@ -5670,19 +5670,19 @@
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="27"/>
       <c r="B44" s="45" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C44" s="45" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D44" s="45" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E44" s="45" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F44" s="45" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G44" s="1"/>
       <c r="H44" s="28"/>
@@ -5690,19 +5690,19 @@
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="27"/>
       <c r="B45" s="46" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C45" s="46" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D45" s="46" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E45" s="46" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F45" s="46" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G45" s="1"/>
       <c r="H45" s="28"/>
@@ -5710,19 +5710,19 @@
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="27"/>
       <c r="B46" s="45" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C46" s="45" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D46" s="45" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E46" s="45" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F46" s="45" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G46" s="1"/>
       <c r="H46" s="28"/>
@@ -5730,19 +5730,19 @@
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="27"/>
       <c r="B47" s="46" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C47" s="46" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D47" s="46" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E47" s="46" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F47" s="46" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G47" s="1"/>
       <c r="H47" s="28"/>
@@ -5750,19 +5750,19 @@
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="27"/>
       <c r="B48" s="45" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C48" s="45" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D48" s="45" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E48" s="45" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F48" s="45" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G48" s="1"/>
       <c r="H48" s="28"/>
@@ -5770,16 +5770,16 @@
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="27"/>
       <c r="B49" s="46" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C49" s="46" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D49" s="46" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E49" s="46" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F49" s="45"/>
       <c r="G49" s="1"/>
@@ -5788,16 +5788,16 @@
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" s="27"/>
       <c r="B50" s="45" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C50" s="45" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D50" s="45" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E50" s="45" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F50" s="45"/>
       <c r="G50" s="1"/>
@@ -5809,7 +5809,7 @@
       <c r="C51" s="51"/>
       <c r="D51" s="45"/>
       <c r="E51" s="46" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F51" s="45"/>
       <c r="G51" s="1"/>
@@ -5821,7 +5821,7 @@
       <c r="C52" s="47"/>
       <c r="D52" s="47"/>
       <c r="E52" s="47" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F52" s="47"/>
       <c r="G52" s="24"/>
@@ -5829,7 +5829,7 @@
     </row>
     <row r="53" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B53" s="30"/>
       <c r="C53" s="31"/>
@@ -5841,7 +5841,7 @@
     </row>
     <row r="54" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B54" s="30"/>
       <c r="C54" s="31"/>
@@ -5907,7 +5907,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B4" s="13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
@@ -5915,7 +5915,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B5" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C5" s="14"/>
       <c r="D5" s="14"/>
@@ -5926,16 +5926,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -6110,7 +6110,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B17" s="7">
         <v>0</v>
@@ -6127,7 +6127,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B18" s="7">
         <v>0</v>
@@ -6144,7 +6144,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B19" s="7">
         <v>0</v>
@@ -6161,7 +6161,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B20" s="7">
         <v>0</v>
@@ -6178,7 +6178,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B21" s="7">
         <v>0</v>
@@ -6195,7 +6195,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B22" s="7">
         <v>0</v>
@@ -6212,7 +6212,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B23" s="7">
         <v>0</v>
@@ -6229,7 +6229,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B24" s="7">
         <v>0</v>
@@ -6246,7 +6246,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B25" s="7">
         <v>0</v>
@@ -6263,7 +6263,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B26" s="7">
         <v>0</v>
@@ -6280,7 +6280,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B27" s="7">
         <v>0</v>
@@ -6297,7 +6297,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B28" s="7">
         <v>0</v>
@@ -6314,7 +6314,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B29" s="7">
         <v>0</v>
@@ -6331,7 +6331,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B30" s="7">
         <v>0</v>
@@ -6348,7 +6348,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B31" s="7">
         <v>0</v>
@@ -6365,7 +6365,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B32" s="7">
         <v>0</v>
@@ -6382,7 +6382,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B33" s="7">
         <v>0</v>
@@ -6432,40 +6432,40 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="B4" s="11" t="s">
         <v>85</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B5" s="11"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="B7" s="11" t="s">
         <v>89</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>91</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -6640,13 +6640,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FEE1B009-7365-4DCB-9085-73227210059D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51A152E0-5019-4E93-8D78-3FBBE8B0DAC8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7002637B-21A6-4FB6-823E-4FBB9FAB0C66}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{585C7326-FAB2-450D-8146-3758A29EF88C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5516004-B1DF-4B73-93AA-7C1AAA34A456}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0BBD66B4-2460-4E7C-8F3F-CAD76004AC7D}"/>
 </file>
</xml_diff>